<commit_message>
fix: formatação e automação das checklists
</commit_message>
<xml_diff>
--- a/CheckLists de autoria/Checklists/Checklist com NCs identificadas e enviadas para o email com data e hora do email.xlsx
+++ b/CheckLists de autoria/Checklists/Checklist com NCs identificadas e enviadas para o email com data e hora do email.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\Engenharia-de-Software-4-periodo\Qualidade de Software\20260904\Checklists\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\PlanoGarantiaQualidade\CheckLists de autoria\Checklists\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FBDEE53A-69BE-47EC-8E58-37680D8C919C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82F22004-6440-47A4-97A6-A2EFB3E00489}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="77">
   <si>
     <t>Avaliação de Processo e Produto - Auditoria de Qualidade</t>
   </si>
@@ -88,9 +88,6 @@
     <t>Nome do projeto avaliado:</t>
   </si>
   <si>
-    <t>Relatório de Teste de Usabilidade do Sistema Web - iFood (+ Documentando_casos_de_teste.xlsx)</t>
-  </si>
-  <si>
     <t>Auditor de QA:</t>
   </si>
   <si>
@@ -164,30 +161,6 @@
   </si>
   <si>
     <t>Total</t>
-  </si>
-  <si>
-    <t>Legenda:</t>
-  </si>
-  <si>
-    <t>• Preencha a coluna 'Resultado' com Conforme / Não Conforme / Não se Aplica para cada item da aba Checklist.</t>
-  </si>
-  <si>
-    <t>• Para itens 'Não Conforme', registre responsável, classificação (Baixa/Média/Alta) e a data/hora de identificação da NC.</t>
-  </si>
-  <si>
-    <t>• A 'Data prevista de resolução' é calculada automaticamente = Data de identificação + prazo (dias) definido na tabela ao lado.</t>
-  </si>
-  <si>
-    <t>• O prazo (dias) de cada classificação é editável (células amarelas); ao alterar, todas as datas previstas recalculam sozinhas.</t>
-  </si>
-  <si>
-    <t>• A conclusão da NC é registrada em 'Data e hora da conclusão da NC' e o 'Status da NC' deve ser atualizado até 'Resolvida' / 'Verificada' / 'Encerrada'.</t>
-  </si>
-  <si>
-    <t>• Aderência = Nº Conforme / (Total de itens - Nº Não se Aplica).</t>
-  </si>
-  <si>
-    <t>• Células com preenchimento amarelo são campos de entrada manual.</t>
   </si>
   <si>
     <t>O relatório descreve o sistema web escolhido, informando nome e finalidade?</t>
@@ -297,6 +270,12 @@
   </si>
   <si>
     <t>Aberta</t>
+  </si>
+  <si>
+    <t>Relatório de Teste de Usabilidade do Sistema Web - iFood</t>
+  </si>
+  <si>
+    <t>4 aulas</t>
   </si>
 </sst>
 </file>
@@ -566,18 +545,29 @@
     <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="10" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -587,21 +577,10 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="22" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="22" fontId="10" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -686,10 +665,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -911,19 +886,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="32"/>
     </row>
     <row r="2" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -950,8 +925,8 @@
       <c r="H2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="40" t="s">
-        <v>81</v>
+      <c r="I2" s="30" t="s">
+        <v>72</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>9</v>
@@ -961,29 +936,29 @@
       </c>
     </row>
     <row r="3" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="28" t="s">
-        <v>53</v>
-      </c>
-      <c r="B3" s="28"/>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="28"/>
-      <c r="G3" s="28"/>
-      <c r="H3" s="28"/>
-      <c r="I3" s="28"/>
-      <c r="J3" s="28"/>
-      <c r="K3" s="28"/>
+      <c r="A3" s="33" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="33"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="33"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="33"/>
+      <c r="G3" s="33"/>
+      <c r="H3" s="33"/>
+      <c r="I3" s="33"/>
+      <c r="J3" s="33"/>
+      <c r="K3" s="33"/>
     </row>
     <row r="4" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>1</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="D4" s="5"/>
       <c r="E4" s="6"/>
@@ -1002,22 +977,22 @@
         <v>2</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="D5" s="39">
+        <v>67</v>
+      </c>
+      <c r="D5" s="29">
         <v>46269.370138888888</v>
       </c>
-      <c r="E5" s="38" t="s">
-        <v>79</v>
+      <c r="E5" s="28" t="s">
+        <v>70</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="G5" s="38" t="s">
-        <v>80</v>
+        <v>35</v>
+      </c>
+      <c r="G5" s="28" t="s">
+        <v>71</v>
       </c>
       <c r="H5" s="5">
         <f>IF(OR($C5&lt;&gt;"Não Conforme",$F5="",$D5=""),"",$D5+INDEX('Resumo e Aderência'!$B$26:$B$28,MATCH($F5,'Resumo e Aderência'!$A$26:$A$28,0))/1440)</f>
@@ -1026,7 +1001,7 @@
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
       <c r="K5" s="4" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1034,10 +1009,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="6"/>
@@ -1056,10 +1031,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="D7" s="5"/>
       <c r="E7" s="6"/>
@@ -1078,10 +1053,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="6"/>
@@ -1096,29 +1071,29 @@
       <c r="K8" s="4"/>
     </row>
     <row r="9" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="28" t="s">
-        <v>54</v>
-      </c>
-      <c r="B9" s="28"/>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28"/>
-      <c r="H9" s="28"/>
-      <c r="I9" s="28"/>
-      <c r="J9" s="28"/>
-      <c r="K9" s="28"/>
+      <c r="A9" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" s="33"/>
+      <c r="C9" s="33"/>
+      <c r="D9" s="33"/>
+      <c r="E9" s="33"/>
+      <c r="F9" s="33"/>
+      <c r="G9" s="33"/>
+      <c r="H9" s="33"/>
+      <c r="I9" s="33"/>
+      <c r="J9" s="33"/>
+      <c r="K9" s="33"/>
     </row>
     <row r="10" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="6"/>
@@ -1137,10 +1112,10 @@
         <v>7</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="D11" s="5"/>
       <c r="E11" s="6"/>
@@ -1159,10 +1134,10 @@
         <v>8</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="D12" s="5"/>
       <c r="E12" s="6"/>
@@ -1181,10 +1156,10 @@
         <v>9</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="D13" s="5"/>
       <c r="E13" s="6"/>
@@ -1203,10 +1178,10 @@
         <v>10</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="6"/>
@@ -1221,29 +1196,29 @@
       <c r="K14" s="4"/>
     </row>
     <row r="15" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="28" t="s">
-        <v>60</v>
-      </c>
-      <c r="B15" s="28"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="28"/>
-      <c r="H15" s="28"/>
-      <c r="I15" s="28"/>
-      <c r="J15" s="28"/>
-      <c r="K15" s="28"/>
+      <c r="A15" s="33" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" s="33"/>
+      <c r="C15" s="33"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="33"/>
+      <c r="F15" s="33"/>
+      <c r="G15" s="33"/>
+      <c r="H15" s="33"/>
+      <c r="I15" s="33"/>
+      <c r="J15" s="33"/>
+      <c r="K15" s="33"/>
     </row>
     <row r="16" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>11</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="D16" s="5"/>
       <c r="E16" s="6"/>
@@ -1262,10 +1237,10 @@
         <v>12</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="D17" s="5"/>
       <c r="E17" s="6"/>
@@ -1284,10 +1259,10 @@
         <v>13</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="D18" s="5"/>
       <c r="E18" s="6"/>
@@ -1306,10 +1281,10 @@
         <v>14</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="D19" s="5"/>
       <c r="E19" s="6"/>
@@ -1325,7 +1300,7 @@
     </row>
     <row r="20" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -1343,10 +1318,10 @@
         <v>15</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="D21" s="5"/>
       <c r="E21" s="6"/>
@@ -1365,10 +1340,10 @@
         <v>16</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="D22" s="5"/>
       <c r="E22" s="6"/>
@@ -1384,7 +1359,7 @@
     </row>
     <row r="23" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -1402,10 +1377,10 @@
         <v>17</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="D24" s="5"/>
       <c r="E24" s="6"/>
@@ -1421,13 +1396,13 @@
     </row>
     <row r="25" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="D25" s="5"/>
       <c r="E25" s="6"/>
@@ -1440,7 +1415,7 @@
     </row>
     <row r="26" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -1458,30 +1433,30 @@
         <v>19</v>
       </c>
       <c r="B27" t="s">
+        <v>64</v>
+      </c>
+      <c r="C27" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="D27" s="31">
+        <v>46269.375</v>
+      </c>
+      <c r="E27" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="C27" s="26" t="s">
-        <v>76</v>
-      </c>
-      <c r="D27" s="41">
-        <v>46269.375</v>
-      </c>
-      <c r="E27" s="26" t="s">
-        <v>82</v>
-      </c>
       <c r="F27" s="26" t="s">
-        <v>37</v>
-      </c>
-      <c r="G27" s="37" t="s">
-        <v>78</v>
-      </c>
-      <c r="H27" s="41">
+        <v>36</v>
+      </c>
+      <c r="G27" s="27" t="s">
+        <v>69</v>
+      </c>
+      <c r="H27" s="31">
         <v>46269.416666666664</v>
       </c>
       <c r="I27" s="24"/>
       <c r="J27" s="24"/>
       <c r="K27" s="26" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1489,9 +1464,11 @@
         <v>20</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C28" s="4"/>
+        <v>65</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>68</v>
+      </c>
       <c r="D28" s="5"/>
       <c r="E28" s="6"/>
       <c r="F28" s="4"/>
@@ -1524,7 +1501,7 @@
     <mergeCell ref="A9:K9"/>
     <mergeCell ref="A15:K15"/>
   </mergeCells>
-  <dataValidations count="3">
+  <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Selecione uma opção da lista." prompt="Selecione o resultado da verificação." sqref="C3:C29" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Conforme,Não Conforme,Não se Aplica"</formula1>
       <formula2>0</formula2>
@@ -1533,9 +1510,12 @@
       <formula1>"Baixa,Média,Alta"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Selecione uma opção da lista." prompt="Selecione o status da não conformidade." sqref="K3:K29" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" error="Selecione uma opção da lista." prompt="Selecione o status da não conformidade." sqref="K3 K9 K15 K20 K23 K26 K29" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"Aberta,Em Resolução,Escalonada,Resolvida,Verificada,Encerrada"</formula1>
       <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K4 K5 K6 K7 K8 K10 K11 K12 K13 K14 K16 K17 K18 K19 K21 K22 K24 K25 K27 K28" xr:uid="{BA0E53C1-157C-424B-A0D5-698C6F27FBC7}">
+      <formula1>"Aberta,Resolvida,Escalonada"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1558,182 +1538,184 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
     </row>
     <row r="4" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
+      <c r="B4" s="35" t="s">
+        <v>75</v>
+      </c>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
     </row>
     <row r="5" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="31" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="35"/>
     </row>
     <row r="6" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="32">
+        <v>16</v>
+      </c>
+      <c r="B6" s="41">
         <v>46269</v>
       </c>
-      <c r="C6" s="32"/>
-      <c r="D6" s="32"/>
-      <c r="E6" s="32"/>
+      <c r="C6" s="41"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="41"/>
     </row>
     <row r="7" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="31"/>
-      <c r="C7" s="31"/>
-      <c r="D7" s="31"/>
-      <c r="E7" s="31"/>
+        <v>17</v>
+      </c>
+      <c r="B7" s="35" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="35"/>
+      <c r="D7" s="35"/>
+      <c r="E7" s="35"/>
     </row>
     <row r="8" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="31" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="31"/>
-      <c r="D8" s="31"/>
-      <c r="E8" s="31"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="35"/>
+      <c r="E8" s="35"/>
     </row>
     <row r="10" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B10" s="8">
-        <f>COUNTA('Checklist - Auditoria'!$B$3:$B$22)</f>
-        <v>16</v>
+        <f>COUNTA('Checklist - Auditoria'!$B$3:$B$28)</f>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B11" s="8">
-        <f>COUNTIF('Checklist - Auditoria'!$C$3:$C$22,"Conforme")</f>
-        <v>15</v>
+        <f>COUNTIF('Checklist - Auditoria'!$C$3:$C$28,"Conforme")</f>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B12" s="8">
-        <f>COUNTIF('Checklist - Auditoria'!$C$3:$C$22,"Não Conforme")</f>
-        <v>1</v>
+        <f>COUNTIF('Checklist - Auditoria'!$C$3:$C$28,"Não Conforme")</f>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B13" s="8">
-        <f>COUNTIF('Checklist - Auditoria'!$C$3:$C$22,"Não se Aplica")</f>
+        <f>COUNTIF('Checklist - Auditoria'!$C$3:$C$28,"Não se Aplica")</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="8">
+        <f>COUNTIFS('Checklist - Auditoria'!$C$3:$C$28,"Não Conforme",'Checklist - Auditoria'!$K$3:$K$28,"&lt;&gt;Resolvida")</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="36" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="8">
-        <f>COUNTIFS('Checklist - Auditoria'!$C$3:$C$22,"Não Conforme",'Checklist - Auditoria'!$K$3:$K$22,"&lt;&gt;Resolvida",'Checklist - Auditoria'!$K$3:$K$22,"&lt;&gt;Verificada",'Checklist - Auditoria'!$K$3:$K$22,"&lt;&gt;Encerrada")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="33" t="s">
+      <c r="B16" s="36"/>
+    </row>
+    <row r="17" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="37">
+        <f>IFERROR(B11/(B10-B13),0)</f>
+        <v>0.9</v>
+      </c>
+      <c r="B17" s="37"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="B16" s="33"/>
-    </row>
-    <row r="17" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="34">
-        <f>IFERROR(B11/(B10-B13),0)</f>
-        <v>0.9375</v>
-      </c>
-      <c r="B17" s="34"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="B19" s="35"/>
+      <c r="B19" s="38"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" s="9" t="s">
         <v>28</v>
-      </c>
-      <c r="B20" s="9" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" s="10" t="s">
         <v>30</v>
-      </c>
-      <c r="B21" s="10" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B22" s="11" t="s">
         <v>32</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C25" s="12" t="s">
         <v>34</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B26" s="14">
         <v>90</v>
@@ -1745,7 +1727,7 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B27" s="14">
         <v>60</v>
@@ -1757,7 +1739,7 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B28" s="14">
         <v>30</v>
@@ -1769,7 +1751,7 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B29" s="17"/>
       <c r="C29" s="18">
@@ -1778,89 +1760,83 @@
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A31" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="A31" s="7"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A32" s="36" t="s">
-        <v>41</v>
-      </c>
-      <c r="B32" s="36"/>
-      <c r="C32" s="36"/>
-      <c r="D32" s="36"/>
-      <c r="E32" s="36"/>
-      <c r="F32" s="36"/>
-      <c r="G32" s="36"/>
+      <c r="A32" s="34"/>
+      <c r="B32" s="34"/>
+      <c r="C32" s="34"/>
+      <c r="D32" s="34"/>
+      <c r="E32" s="34"/>
+      <c r="F32" s="34"/>
+      <c r="G32" s="34"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A33" s="36" t="s">
-        <v>42</v>
-      </c>
-      <c r="B33" s="36"/>
-      <c r="C33" s="36"/>
-      <c r="D33" s="36"/>
-      <c r="E33" s="36"/>
-      <c r="F33" s="36"/>
-      <c r="G33" s="36"/>
+      <c r="A33" s="34"/>
+      <c r="B33" s="34"/>
+      <c r="C33" s="34"/>
+      <c r="D33" s="34"/>
+      <c r="E33" s="34"/>
+      <c r="F33" s="34"/>
+      <c r="G33" s="34"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A34" s="36" t="s">
-        <v>43</v>
-      </c>
-      <c r="B34" s="36"/>
-      <c r="C34" s="36"/>
-      <c r="D34" s="36"/>
-      <c r="E34" s="36"/>
-      <c r="F34" s="36"/>
-      <c r="G34" s="36"/>
+      <c r="A34" s="34"/>
+      <c r="B34" s="34"/>
+      <c r="C34" s="34"/>
+      <c r="D34" s="34"/>
+      <c r="E34" s="34"/>
+      <c r="F34" s="34"/>
+      <c r="G34" s="34"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A35" s="36" t="s">
-        <v>44</v>
-      </c>
-      <c r="B35" s="36"/>
-      <c r="C35" s="36"/>
-      <c r="D35" s="36"/>
-      <c r="E35" s="36"/>
-      <c r="F35" s="36"/>
-      <c r="G35" s="36"/>
+      <c r="A35" s="34"/>
+      <c r="B35" s="34"/>
+      <c r="C35" s="34"/>
+      <c r="D35" s="34"/>
+      <c r="E35" s="34"/>
+      <c r="F35" s="34"/>
+      <c r="G35" s="34"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A36" s="36" t="s">
-        <v>45</v>
-      </c>
-      <c r="B36" s="36"/>
-      <c r="C36" s="36"/>
-      <c r="D36" s="36"/>
-      <c r="E36" s="36"/>
-      <c r="F36" s="36"/>
-      <c r="G36" s="36"/>
+      <c r="A36" s="34"/>
+      <c r="B36" s="34"/>
+      <c r="C36" s="34"/>
+      <c r="D36" s="34"/>
+      <c r="E36" s="34"/>
+      <c r="F36" s="34"/>
+      <c r="G36" s="34"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A37" s="36" t="s">
-        <v>46</v>
-      </c>
-      <c r="B37" s="36"/>
-      <c r="C37" s="36"/>
-      <c r="D37" s="36"/>
-      <c r="E37" s="36"/>
-      <c r="F37" s="36"/>
-      <c r="G37" s="36"/>
+      <c r="A37" s="34"/>
+      <c r="B37" s="34"/>
+      <c r="C37" s="34"/>
+      <c r="D37" s="34"/>
+      <c r="E37" s="34"/>
+      <c r="F37" s="34"/>
+      <c r="G37" s="34"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A38" s="36" t="s">
-        <v>47</v>
-      </c>
-      <c r="B38" s="36"/>
-      <c r="C38" s="36"/>
-      <c r="D38" s="36"/>
-      <c r="E38" s="36"/>
-      <c r="F38" s="36"/>
-      <c r="G38" s="36"/>
+      <c r="A38" s="34"/>
+      <c r="B38" s="34"/>
+      <c r="C38" s="34"/>
+      <c r="D38" s="34"/>
+      <c r="E38" s="34"/>
+      <c r="F38" s="34"/>
+      <c r="G38" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A19:B19"/>
     <mergeCell ref="A37:G37"/>
     <mergeCell ref="A38:G38"/>
     <mergeCell ref="A32:G32"/>
@@ -1868,16 +1844,6 @@
     <mergeCell ref="A34:G34"/>
     <mergeCell ref="A35:G35"/>
     <mergeCell ref="A36:G36"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B6:E6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>